<commit_message>
docs: 同步文档内容 (2026-04-26 22:14:35)
</commit_message>
<xml_diff>
--- a/downloads/excel/team_member.xlsx
+++ b/downloads/excel/team_member.xlsx
@@ -1,297 +1,190 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15600"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="15600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="member" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="member" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
-  <si>
-    <t>昵称</t>
-  </si>
-  <si>
-    <t>邮箱</t>
-  </si>
-  <si>
-    <t>手机</t>
-  </si>
-  <si>
-    <t>工号</t>
-  </si>
-  <si>
-    <t>职位</t>
-  </si>
-  <si>
-    <t>部门</t>
-  </si>
-  <si>
-    <t>座位号</t>
-  </si>
-  <si>
-    <t>分机号</t>
-  </si>
-  <si>
-    <t>test0</t>
-  </si>
-  <si>
-    <t>100@email.com</t>
-  </si>
-  <si>
-    <t>CEO</t>
-  </si>
-  <si>
-    <t>测试部门</t>
-  </si>
-  <si>
-    <t>test1</t>
-  </si>
-  <si>
-    <t>101@email.com</t>
-  </si>
-  <si>
-    <t>CTO</t>
-  </si>
-  <si>
-    <t>设计部门</t>
-  </si>
-  <si>
-    <t>test2</t>
-  </si>
-  <si>
-    <t>102@email.com</t>
-  </si>
-  <si>
-    <t>部门经理</t>
-  </si>
-  <si>
-    <t>开发部门</t>
-  </si>
-  <si>
-    <t>test3</t>
-  </si>
-  <si>
-    <t>103@email.com</t>
-  </si>
-  <si>
-    <t>运营部门</t>
-  </si>
-  <si>
-    <t>test4</t>
-  </si>
-  <si>
-    <t>104@email.com</t>
-  </si>
-  <si>
-    <t>员工</t>
-  </si>
-  <si>
-    <t>test5</t>
-  </si>
-  <si>
-    <t>105@email.com</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="22">
     <font>
-      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color indexed="8"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="34">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -612,164 +505,165 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="6"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="6"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1015,7 +909,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -1024,7 +918,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
       <tableStyleElement type="headerRow" dxfId="16"/>
       <tableStyleElement type="totalRow" dxfId="15"/>
       <tableStyleElement type="firstRowStripe" dxfId="14"/>
@@ -1037,11 +931,74 @@
       <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1301,206 +1258,304 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="6"/>
   <cols>
-    <col min="1" max="8" width="20" customWidth="1"/>
+    <col width="20" customWidth="1" style="5" min="1" max="8"/>
+    <col width="28" customWidth="1" style="5" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" spans="1:8">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="21" customHeight="1" s="5">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>昵称</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>邮箱</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>手机</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>工号</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>职位</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>部门</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>座位号</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>分机号</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>可登录平台</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" customFormat="1" s="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>test0</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>100@email.com</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>18888888000</v>
+      </c>
+      <c r="D2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>测试部门</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3" customFormat="1" s="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>101@email.com</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>18800000001</v>
+      </c>
+      <c r="D3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>设计部门</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" customFormat="1" s="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>test2</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>102@email.com</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>18800000002</v>
+      </c>
+      <c r="D4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>部门经理</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>开发部门</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>admin,desktop</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" customFormat="1" s="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>test3</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>103@email.com</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>18800000003</v>
+      </c>
+      <c r="D5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>部门经理</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>运营部门</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>notebase,workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" customFormat="1" s="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>test4</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>104@email.com</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>18800000004</v>
+      </c>
+      <c r="D6" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>员工</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>运营部门</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>call,callAdmin</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" customFormat="1" s="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>test5</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>105@email.com</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>18800000005</v>
+      </c>
+      <c r="D7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" s="1" customFormat="1" spans="1:8">
-      <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="1">
-        <v>18888888000</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="1">
-        <v>0</v>
-      </c>
-      <c r="H2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" s="1" customFormat="1" spans="1:8">
-      <c r="A3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="1">
-        <v>18800000001</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="1">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" s="1" customFormat="1" spans="1:8">
-      <c r="A4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="1">
-        <v>18800000002</v>
-      </c>
-      <c r="D4" s="1">
-        <v>2</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="1">
-        <v>2</v>
-      </c>
-      <c r="H4" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" s="1" customFormat="1" spans="1:8">
-      <c r="A5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="1">
-        <v>18800000003</v>
-      </c>
-      <c r="D5" s="1">
-        <v>3</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="1">
-        <v>3</v>
-      </c>
-      <c r="H5" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" s="1" customFormat="1" spans="1:8">
-      <c r="A6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="1">
-        <v>18800000004</v>
-      </c>
-      <c r="D6" s="1">
-        <v>4</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="1">
-        <v>4</v>
-      </c>
-      <c r="H6" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" s="1" customFormat="1" spans="1:8">
-      <c r="A7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="1">
-        <v>18800000005</v>
-      </c>
-      <c r="D7" s="1">
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>员工</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>运营部门</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="1">
+      <c r="H7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="1">
-        <v>5</v>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="100@email.com" tooltip="mailto:100@email.com"/>
-    <hyperlink ref="B3" r:id="rId2" display="101@email.com" tooltip="mailto:101@email.com"/>
-    <hyperlink ref="B4" r:id="rId3" display="102@email.com" tooltip="mailto:102@email.com"/>
-    <hyperlink ref="B5" r:id="rId4" display="103@email.com"/>
-    <hyperlink ref="B6" r:id="rId5" display="104@email.com"/>
-    <hyperlink ref="B7" r:id="rId6" display="105@email.com"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" tooltip="mailto:100@email.com" display="100@email.com" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" tooltip="mailto:101@email.com" display="101@email.com" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" tooltip="mailto:102@email.com" display="102@email.com" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" display="103@email.com" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" display="104@email.com" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" display="105@email.com" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>